<commit_message>
Update Chapter 5, test plan, test cases and results
</commit_message>
<xml_diff>
--- a/06_Testing_Results_and_Evaluation/Test_Cases_and_Results.xlsx
+++ b/06_Testing_Results_and_Evaluation/Test_Cases_and_Results.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ctutrainingsolutionspt-my.sharepoint.com/personal/lusukama_selemani_ctutraining_co_za/Documents/Documents/POES-LUSUKAMA/Research-2026/Capstone_Project_Pack_with_CTU_Logo/Capstone_Project_Pack/06_Testing_Results_and_Evaluation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sihle Kayise\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{CEC173AF-77E1-48A0-B51B-C576C11049EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76BDD8FA-5754-45B1-8952-8D827E804FC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tracker" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tracker!$A$3:$L$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tracker!$A$3:$L$100</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="120">
   <si>
     <t>SOFTWARE TEST CASES &amp; RESULTS</t>
   </si>
@@ -62,13 +62,334 @@
   </si>
   <si>
     <t>Evidence</t>
+  </si>
+  <si>
+    <t>TC-001</t>
+  </si>
+  <si>
+    <t>REQ-001</t>
+  </si>
+  <si>
+    <t>Student Login</t>
+  </si>
+  <si>
+    <t>Student account exists and system is online</t>
+  </si>
+  <si>
+    <t>1. Open login page. 2. Enter valid student credentials. 3. Click Login.</t>
+  </si>
+  <si>
+    <t>Valid student username and password</t>
+  </si>
+  <si>
+    <t>Student should successfully log in and be redirected to dashboard.</t>
+  </si>
+  <si>
+    <t>Student logged in successfully and dashboard displayed.</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Sihle Kayise</t>
+  </si>
+  <si>
+    <t>TC-002</t>
+  </si>
+  <si>
+    <t>REQ-002</t>
+  </si>
+  <si>
+    <t>Student Dashboard</t>
+  </si>
+  <si>
+    <t>Student is logged in</t>
+  </si>
+  <si>
+    <t>1. Log in as student. 2. View dashboard.</t>
+  </si>
+  <si>
+    <t>Student account</t>
+  </si>
+  <si>
+    <t>Dashboard should load and all functions should be accessible.</t>
+  </si>
+  <si>
+    <t>Dashboard appeared and worked correctly.</t>
+  </si>
+  <si>
+    <t>TC-003</t>
+  </si>
+  <si>
+    <t>REQ-003</t>
+  </si>
+  <si>
+    <t>View Existing Logbook Entry</t>
+  </si>
+  <si>
+    <t>Student has an existing logbook entry</t>
+  </si>
+  <si>
+    <t>1. Open dashboard. 2. Click on an existing entry date.</t>
+  </si>
+  <si>
+    <t>Existing logbook entry</t>
+  </si>
+  <si>
+    <t>Selected entry details should open successfully.</t>
+  </si>
+  <si>
+    <t>Entry displayed successfully.</t>
+  </si>
+  <si>
+    <t>TC-004</t>
+  </si>
+  <si>
+    <t>REQ-004</t>
+  </si>
+  <si>
+    <t>Back to Logbook Navigation</t>
+  </si>
+  <si>
+    <t>Student is viewing a logbook entry</t>
+  </si>
+  <si>
+    <t>1. Open an entry. 2. Click "Back to Logbook".</t>
+  </si>
+  <si>
+    <t>Existing entry</t>
+  </si>
+  <si>
+    <t>User should be redirected to Logbook Dashboard.</t>
+  </si>
+  <si>
+    <t>Redirected successfully to Logbook Dashboard.</t>
+  </si>
+  <si>
+    <t>TC-005</t>
+  </si>
+  <si>
+    <t>REQ-005</t>
+  </si>
+  <si>
+    <t>Create New Logbook Entry</t>
+  </si>
+  <si>
+    <t>1. Click "New Entry". 2. Complete all fields. 3. Submit entry.</t>
+  </si>
+  <si>
+    <t>Logbook information (date, activities, hours worked, comments)</t>
+  </si>
+  <si>
+    <t>New entry form should open and accept user input.</t>
+  </si>
+  <si>
+    <t>New entry created successfully and all fields were functional.</t>
+  </si>
+  <si>
+    <t>TC-006</t>
+  </si>
+  <si>
+    <t>REQ-006</t>
+  </si>
+  <si>
+    <t>Save Logbook Entry</t>
+  </si>
+  <si>
+    <t>New logbook entry has been completed</t>
+  </si>
+  <si>
+    <t>1. Fill in entry form. 2. Click "Save Entry".</t>
+  </si>
+  <si>
+    <t>Completed logbook details</t>
+  </si>
+  <si>
+    <t>Entry should save successfully and appear on dashboard.</t>
+  </si>
+  <si>
+    <t>Entry saved successfully and displayed on logbook dashboard.</t>
+  </si>
+  <si>
+    <t>TC-007</t>
+  </si>
+  <si>
+    <t>REQ-007</t>
+  </si>
+  <si>
+    <t>Student Sign Out</t>
+  </si>
+  <si>
+    <t>1. Click "Sign Out".</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>User should be logged out and redirected to login page.</t>
+  </si>
+  <si>
+    <t>Redirected to login page successfully.</t>
+  </si>
+  <si>
+    <t>TC-008</t>
+  </si>
+  <si>
+    <t>REQ-008</t>
+  </si>
+  <si>
+    <t>Coordinator Login</t>
+  </si>
+  <si>
+    <t>Coordinator account exists</t>
+  </si>
+  <si>
+    <t>1. Open login page. 2. Enter valid coordinator credentials. 3. Click Login.</t>
+  </si>
+  <si>
+    <t>Valid coordinator username and password</t>
+  </si>
+  <si>
+    <t>Coordinator should successfully log in.</t>
+  </si>
+  <si>
+    <t>Coordinator signed in successfully.</t>
+  </si>
+  <si>
+    <t>TC-009</t>
+  </si>
+  <si>
+    <t>REQ-009</t>
+  </si>
+  <si>
+    <t>Coordinator Dashboard</t>
+  </si>
+  <si>
+    <t>Coordinator is logged in</t>
+  </si>
+  <si>
+    <t>1. Log in as coordinator. 2. View dashboard.</t>
+  </si>
+  <si>
+    <t>Uploaded student logbook entries</t>
+  </si>
+  <si>
+    <t>Dashboard should display students who submitted entries.</t>
+  </si>
+  <si>
+    <t>Submitted student entries were visible.</t>
+  </si>
+  <si>
+    <t>TC-010</t>
+  </si>
+  <si>
+    <t>REQ-010</t>
+  </si>
+  <si>
+    <t>Coordinator Sign Out</t>
+  </si>
+  <si>
+    <t>User should be redirected to login page.</t>
+  </si>
+  <si>
+    <t>Redirected successfully to login page.</t>
+  </si>
+  <si>
+    <t>TC-011</t>
+  </si>
+  <si>
+    <t>TC-012</t>
+  </si>
+  <si>
+    <t>REQ-012</t>
+  </si>
+  <si>
+    <t>Student Login with Invalid Credentials</t>
+  </si>
+  <si>
+    <t>Student login page is accessible</t>
+  </si>
+  <si>
+    <t>1. Open login page. 2. Enter invalid username and/or password. 3. Click Login.</t>
+  </si>
+  <si>
+    <t>Invalid username/password</t>
+  </si>
+  <si>
+    <t>System should display an error message and deny access.</t>
+  </si>
+  <si>
+    <t>Error message displayed and login was unsuccessful.</t>
+  </si>
+  <si>
+    <t>TC-013</t>
+  </si>
+  <si>
+    <t>TC-014</t>
+  </si>
+  <si>
+    <t>REQ-014</t>
+  </si>
+  <si>
+    <t>Save Logbook Entry with Required Fields Empty</t>
+  </si>
+  <si>
+    <t>Student is logged in and on the New Entry page</t>
+  </si>
+  <si>
+    <t>1. Click "New Entry". 2. Leave one or more required fields blank. 3. Click "Save Entry".</t>
+  </si>
+  <si>
+    <t>Incomplete logbook entry</t>
+  </si>
+  <si>
+    <t>System should validate input and prevent saving until all required fields are completed.</t>
+  </si>
+  <si>
+    <t>Validation message displayed and entry was not saved.</t>
+  </si>
+  <si>
+    <t>REQ-015</t>
+  </si>
+  <si>
+    <t>Coordinator Login with Invalid Credentials</t>
+  </si>
+  <si>
+    <t>Coordinator login page is accessible</t>
+  </si>
+  <si>
+    <t>1. Enter incorrect login credentials. 2. Click Login.</t>
+  </si>
+  <si>
+    <t>Invalid coordinator username/password</t>
+  </si>
+  <si>
+    <t>REQ-017</t>
+  </si>
+  <si>
+    <t>Verify Saved Data After Logout and Login</t>
+  </si>
+  <si>
+    <t>Student has previously saved a logbook entry</t>
+  </si>
+  <si>
+    <t>1. Create and save a logbook entry. 2. Sign out. 3. Sign back in. 4. Open the logbook dashboard.</t>
+  </si>
+  <si>
+    <t>Previously saved logbook entry</t>
+  </si>
+  <si>
+    <t>Saved entry should still be available on the dashboard.</t>
+  </si>
+  <si>
+    <t>Saved entry remained visible after logging back in.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,6 +407,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -106,7 +433,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -132,17 +459,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFE6E6E6"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFE6E6E6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFE6E6E6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFE6E6E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -448,8 +796,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L53"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:L50"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -464,23 +812,23 @@
     <col min="12" max="12" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+    </row>
+    <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -518,203 +866,510 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="4">
+        <v>46317</v>
+      </c>
+      <c r="L4" s="3"/>
+    </row>
+    <row r="5" spans="1:12" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5" s="4">
+        <v>46317</v>
+      </c>
+      <c r="L5" s="3"/>
+    </row>
+    <row r="6" spans="1:12" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" s="4">
+        <v>46317</v>
+      </c>
+      <c r="L6" s="3"/>
+    </row>
+    <row r="7" spans="1:12" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" s="4">
+        <v>46317</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K8" s="4">
+        <v>46317</v>
+      </c>
+      <c r="L8" s="3"/>
+    </row>
+    <row r="9" spans="1:12" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K9" s="4">
+        <v>46317</v>
+      </c>
+      <c r="L9" s="3"/>
+    </row>
+    <row r="10" spans="1:12" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K10" s="4">
+        <v>46317</v>
+      </c>
+      <c r="L10" s="3"/>
+    </row>
+    <row r="11" spans="1:12" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K11" s="4">
+        <v>46317</v>
+      </c>
+      <c r="L11" s="3"/>
+    </row>
+    <row r="12" spans="1:12" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K12" s="4">
+        <v>46317</v>
+      </c>
+      <c r="L12" s="3"/>
+    </row>
+    <row r="13" spans="1:12" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K13" s="4">
+        <v>46317</v>
+      </c>
+      <c r="L13" s="3"/>
+    </row>
+    <row r="14" spans="1:12" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K14" s="4">
+        <v>46317</v>
+      </c>
+      <c r="L14" s="3"/>
+    </row>
+    <row r="15" spans="1:12" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K15" s="4">
+        <v>46317</v>
+      </c>
+      <c r="L15" s="3"/>
+    </row>
+    <row r="16" spans="1:12" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K16" s="4">
+        <v>46317</v>
+      </c>
+      <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="1:12" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K17" s="4">
+        <v>46317</v>
+      </c>
+      <c r="L17" s="3"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -728,7 +1383,7 @@
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -742,7 +1397,7 @@
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -756,7 +1411,7 @@
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -770,7 +1425,7 @@
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -784,7 +1439,7 @@
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -798,7 +1453,7 @@
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -812,7 +1467,7 @@
       <c r="K24" s="2"/>
       <c r="L24" s="2"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -826,7 +1481,7 @@
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -840,7 +1495,7 @@
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -854,7 +1509,7 @@
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -868,7 +1523,7 @@
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -882,7 +1537,7 @@
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -896,7 +1551,7 @@
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -910,7 +1565,7 @@
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -924,7 +1579,7 @@
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -938,7 +1593,7 @@
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -952,7 +1607,7 @@
       <c r="K34" s="2"/>
       <c r="L34" s="2"/>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -966,7 +1621,7 @@
       <c r="K35" s="2"/>
       <c r="L35" s="2"/>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -980,7 +1635,7 @@
       <c r="K36" s="2"/>
       <c r="L36" s="2"/>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -994,7 +1649,7 @@
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -1008,7 +1663,7 @@
       <c r="K38" s="2"/>
       <c r="L38" s="2"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -1022,7 +1677,7 @@
       <c r="K39" s="2"/>
       <c r="L39" s="2"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -1036,7 +1691,7 @@
       <c r="K40" s="2"/>
       <c r="L40" s="2"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -1050,7 +1705,7 @@
       <c r="K41" s="2"/>
       <c r="L41" s="2"/>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -1064,7 +1719,7 @@
       <c r="K42" s="2"/>
       <c r="L42" s="2"/>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -1078,7 +1733,7 @@
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -1092,7 +1747,7 @@
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -1106,7 +1761,7 @@
       <c r="K45" s="2"/>
       <c r="L45" s="2"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -1120,7 +1775,7 @@
       <c r="K46" s="2"/>
       <c r="L46" s="2"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -1134,7 +1789,7 @@
       <c r="K47" s="2"/>
       <c r="L47" s="2"/>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -1148,7 +1803,7 @@
       <c r="K48" s="2"/>
       <c r="L48" s="2"/>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -1162,7 +1817,7 @@
       <c r="K49" s="2"/>
       <c r="L49" s="2"/>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -1176,55 +1831,13 @@
       <c r="K50" s="2"/>
       <c r="L50" s="2"/>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A51" s="2"/>
-      <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="2"/>
-      <c r="H51" s="2"/>
-      <c r="I51" s="2"/>
-      <c r="J51" s="2"/>
-      <c r="K51" s="2"/>
-      <c r="L51" s="2"/>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-      <c r="G52" s="2"/>
-      <c r="H52" s="2"/>
-      <c r="I52" s="2"/>
-      <c r="J52" s="2"/>
-      <c r="K52" s="2"/>
-      <c r="L52" s="2"/>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
-      <c r="G53" s="2"/>
-      <c r="H53" s="2"/>
-      <c r="I53" s="2"/>
-      <c r="J53" s="2"/>
-      <c r="K53" s="2"/>
-      <c r="L53" s="2"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A3:L103" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A3:L100" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="I4:I53" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I18:I50" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not Run,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>